<commit_message>
run code and data updates
</commit_message>
<xml_diff>
--- a/data/excel/kof_indicator_business_situation.xlsx
+++ b/data/excel/kof_indicator_business_situation.xlsx
@@ -6468,7 +6468,7 @@
         <v>17</v>
       </c>
       <c r="J518">
-        <v>-10.9</v>
+        <v>-10.89</v>
       </c>
     </row>
     <row r="519">
@@ -6577,7 +6577,7 @@
         <v>2016-07</v>
       </c>
       <c r="B523">
-        <v>46.55</v>
+        <v>46.54</v>
       </c>
       <c r="C523">
         <v>22.28</v>
@@ -6866,7 +6866,7 @@
         <v>2017-06</v>
       </c>
       <c r="B534">
-        <v>47.32</v>
+        <v>47.31</v>
       </c>
       <c r="C534">
         <v>28.95</v>
@@ -7045,7 +7045,7 @@
         <v>2018-01</v>
       </c>
       <c r="B541">
-        <v>46.89</v>
+        <v>46.9</v>
       </c>
       <c r="C541">
         <v>30.75</v>
@@ -7092,7 +7092,7 @@
         <v>38.6</v>
       </c>
       <c r="J542">
-        <v>21.16</v>
+        <v>21.17</v>
       </c>
     </row>
     <row r="543">
@@ -7412,7 +7412,7 @@
         <v>2019-03</v>
       </c>
       <c r="B555">
-        <v>52.89</v>
+        <v>52.9</v>
       </c>
       <c r="C555">
         <v>29.43</v>
@@ -7490,7 +7490,7 @@
         <v>2019-06</v>
       </c>
       <c r="B558">
-        <v>55.79</v>
+        <v>55.78</v>
       </c>
       <c r="C558">
         <v>34.32</v>
@@ -7513,7 +7513,7 @@
         <v>2019-07</v>
       </c>
       <c r="B559">
-        <v>51.82</v>
+        <v>51.81</v>
       </c>
       <c r="C559">
         <v>34.24</v>
@@ -7623,7 +7623,7 @@
         <v>2019-11</v>
       </c>
       <c r="B563">
-        <v>55.68</v>
+        <v>55.69</v>
       </c>
       <c r="C563">
         <v>33</v>
@@ -7736,7 +7736,7 @@
         <v>48.74</v>
       </c>
       <c r="C567">
-        <v>32.58</v>
+        <v>32.59</v>
       </c>
       <c r="D567">
         <v>15.85</v>
@@ -7843,7 +7843,7 @@
         <v>2020-07</v>
       </c>
       <c r="B571">
-        <v>35.3</v>
+        <v>35.29</v>
       </c>
       <c r="C571">
         <v>12.77</v>
@@ -7927,7 +7927,7 @@
         <v>2020-10</v>
       </c>
       <c r="B574">
-        <v>38.1</v>
+        <v>38.11</v>
       </c>
       <c r="C574">
         <v>20.28</v>
@@ -7985,7 +7985,7 @@
         <v>2020-12</v>
       </c>
       <c r="B576">
-        <v>39.66</v>
+        <v>39.67</v>
       </c>
       <c r="C576">
         <v>21.36</v>
@@ -8014,7 +8014,7 @@
         <v>40.41</v>
       </c>
       <c r="C577">
-        <v>23.47</v>
+        <v>23.46</v>
       </c>
       <c r="D577">
         <v>0.99</v>
@@ -8043,10 +8043,10 @@
         <v>2021-02</v>
       </c>
       <c r="B578">
-        <v>36.47</v>
+        <v>36.48</v>
       </c>
       <c r="C578">
-        <v>23.45</v>
+        <v>23.44</v>
       </c>
       <c r="D578">
         <v>-0.09</v>
@@ -8087,7 +8087,7 @@
         <v>39.88</v>
       </c>
       <c r="J579">
-        <v>4.32</v>
+        <v>4.33</v>
       </c>
     </row>
     <row r="580">
@@ -8095,7 +8095,7 @@
         <v>2021-04</v>
       </c>
       <c r="B580">
-        <v>44.94</v>
+        <v>44.93</v>
       </c>
       <c r="C580">
         <v>31.83</v>
@@ -8119,7 +8119,7 @@
         <v>23.3</v>
       </c>
       <c r="J580">
-        <v>20.82</v>
+        <v>20.81</v>
       </c>
     </row>
     <row r="581">
@@ -8127,7 +8127,7 @@
         <v>2021-05</v>
       </c>
       <c r="B581">
-        <v>47.59</v>
+        <v>47.58</v>
       </c>
       <c r="C581">
         <v>34.58</v>
@@ -8156,7 +8156,7 @@
         <v>49.49</v>
       </c>
       <c r="C582">
-        <v>33.48</v>
+        <v>33.49</v>
       </c>
       <c r="D582">
         <v>16.86</v>
@@ -8179,7 +8179,7 @@
         <v>2021-07</v>
       </c>
       <c r="B583">
-        <v>53.49</v>
+        <v>53.48</v>
       </c>
       <c r="C583">
         <v>37.04</v>
@@ -8263,7 +8263,7 @@
         <v>2021-10</v>
       </c>
       <c r="B586">
-        <v>54.51</v>
+        <v>54.53</v>
       </c>
       <c r="C586">
         <v>38.82</v>
@@ -8295,10 +8295,10 @@
         <v>2021-11</v>
       </c>
       <c r="B587">
-        <v>55.75</v>
+        <v>55.76</v>
       </c>
       <c r="C587">
-        <v>39.15</v>
+        <v>39.14</v>
       </c>
       <c r="D587">
         <v>29.89</v>
@@ -8313,7 +8313,7 @@
         <v>44.84</v>
       </c>
       <c r="J587">
-        <v>31.55</v>
+        <v>31.56</v>
       </c>
     </row>
     <row r="588">
@@ -8324,7 +8324,7 @@
         <v>56.23</v>
       </c>
       <c r="C588">
-        <v>40.43</v>
+        <v>40.42</v>
       </c>
       <c r="D588">
         <v>29.47</v>
@@ -8350,7 +8350,7 @@
         <v>57.27</v>
       </c>
       <c r="C589">
-        <v>40.74</v>
+        <v>40.73</v>
       </c>
       <c r="D589">
         <v>28.23</v>
@@ -8382,7 +8382,7 @@
         <v>58.58</v>
       </c>
       <c r="C590">
-        <v>42.77</v>
+        <v>42.75</v>
       </c>
       <c r="D590">
         <v>31.97</v>
@@ -8408,7 +8408,7 @@
         <v>57.22</v>
       </c>
       <c r="C591">
-        <v>40.8</v>
+        <v>40.79</v>
       </c>
       <c r="D591">
         <v>29.9</v>
@@ -8431,10 +8431,10 @@
         <v>2022-04</v>
       </c>
       <c r="B592">
-        <v>57.28</v>
+        <v>57.27</v>
       </c>
       <c r="C592">
-        <v>40.98</v>
+        <v>41.02</v>
       </c>
       <c r="D592">
         <v>32.5</v>
@@ -8463,7 +8463,7 @@
         <v>2022-05</v>
       </c>
       <c r="B593">
-        <v>56.51</v>
+        <v>56.5</v>
       </c>
       <c r="C593">
         <v>40.68</v>
@@ -8492,7 +8492,7 @@
         <v>52.49</v>
       </c>
       <c r="C594">
-        <v>39.64</v>
+        <v>39.65</v>
       </c>
       <c r="D594">
         <v>31.98</v>
@@ -8515,7 +8515,7 @@
         <v>2022-07</v>
       </c>
       <c r="B595">
-        <v>50.02</v>
+        <v>50.01</v>
       </c>
       <c r="C595">
         <v>43.66</v>
@@ -8539,7 +8539,7 @@
         <v>51.77</v>
       </c>
       <c r="J595">
-        <v>30.02</v>
+        <v>30.01</v>
       </c>
     </row>
     <row r="596">
@@ -8550,7 +8550,7 @@
         <v>53.44</v>
       </c>
       <c r="C596">
-        <v>42.08</v>
+        <v>42.09</v>
       </c>
       <c r="D596">
         <v>27.6</v>
@@ -8599,7 +8599,7 @@
         <v>2022-10</v>
       </c>
       <c r="B598">
-        <v>51.64</v>
+        <v>51.67</v>
       </c>
       <c r="C598">
         <v>44.14</v>
@@ -8631,10 +8631,10 @@
         <v>2022-11</v>
       </c>
       <c r="B599">
-        <v>48.64</v>
+        <v>48.65</v>
       </c>
       <c r="C599">
-        <v>44.77</v>
+        <v>44.76</v>
       </c>
       <c r="D599">
         <v>24.19</v>
@@ -8657,10 +8657,10 @@
         <v>2022-12</v>
       </c>
       <c r="B600">
-        <v>52.94</v>
+        <v>52.95</v>
       </c>
       <c r="C600">
-        <v>47.31</v>
+        <v>47.3</v>
       </c>
       <c r="D600">
         <v>25.22</v>
@@ -8675,7 +8675,7 @@
         <v>27.85</v>
       </c>
       <c r="J600">
-        <v>18.91</v>
+        <v>18.92</v>
       </c>
     </row>
     <row r="601">
@@ -8683,10 +8683,10 @@
         <v>2023-01</v>
       </c>
       <c r="B601">
-        <v>54.7</v>
+        <v>54.71</v>
       </c>
       <c r="C601">
-        <v>48.89</v>
+        <v>48.87</v>
       </c>
       <c r="D601">
         <v>29.61</v>
@@ -8715,10 +8715,10 @@
         <v>2023-02</v>
       </c>
       <c r="B602">
-        <v>54.66</v>
+        <v>54.67</v>
       </c>
       <c r="C602">
-        <v>47.27</v>
+        <v>47.24</v>
       </c>
       <c r="D602">
         <v>27.84</v>
@@ -8733,7 +8733,7 @@
         <v>36.74</v>
       </c>
       <c r="J602">
-        <v>18.73</v>
+        <v>18.74</v>
       </c>
     </row>
     <row r="603">
@@ -8741,10 +8741,10 @@
         <v>2023-03</v>
       </c>
       <c r="B603">
-        <v>55.64</v>
+        <v>55.6</v>
       </c>
       <c r="C603">
-        <v>48.63</v>
+        <v>48.61</v>
       </c>
       <c r="D603">
         <v>28.28</v>
@@ -8770,7 +8770,7 @@
         <v>55.91</v>
       </c>
       <c r="C604">
-        <v>46.26</v>
+        <v>46.35</v>
       </c>
       <c r="D604">
         <v>24.18</v>
@@ -8791,7 +8791,7 @@
         <v>37.79</v>
       </c>
       <c r="J604">
-        <v>7.86</v>
+        <v>7.85</v>
       </c>
     </row>
     <row r="605">
@@ -8799,10 +8799,10 @@
         <v>2023-05</v>
       </c>
       <c r="B605">
-        <v>50.18</v>
+        <v>50.17</v>
       </c>
       <c r="C605">
-        <v>40.39</v>
+        <v>40.4</v>
       </c>
       <c r="D605">
         <v>22.76</v>
@@ -8817,7 +8817,7 @@
         <v>42.49</v>
       </c>
       <c r="J605">
-        <v>-0.14</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="606">
@@ -8825,10 +8825,10 @@
         <v>2023-06</v>
       </c>
       <c r="B606">
-        <v>56.17</v>
+        <v>56.16</v>
       </c>
       <c r="C606">
-        <v>45.11</v>
+        <v>45.12</v>
       </c>
       <c r="D606">
         <v>21.57</v>
@@ -8851,7 +8851,7 @@
         <v>2023-07</v>
       </c>
       <c r="B607">
-        <v>53.81</v>
+        <v>53.8</v>
       </c>
       <c r="C607">
         <v>42.93</v>
@@ -8875,7 +8875,7 @@
         <v>21.34</v>
       </c>
       <c r="J607">
-        <v>-5.98</v>
+        <v>-5.99</v>
       </c>
     </row>
     <row r="608">
@@ -8912,7 +8912,7 @@
         <v>54.34</v>
       </c>
       <c r="C609">
-        <v>43.4</v>
+        <v>43.39</v>
       </c>
       <c r="D609">
         <v>16.91</v>
@@ -8927,7 +8927,7 @@
         <v>41.5</v>
       </c>
       <c r="J609">
-        <v>-4.21</v>
+        <v>-4.22</v>
       </c>
     </row>
     <row r="610">
@@ -8935,10 +8935,10 @@
         <v>2023-10</v>
       </c>
       <c r="B610">
-        <v>57.44</v>
+        <v>57.48</v>
       </c>
       <c r="C610">
-        <v>44.41</v>
+        <v>44.4</v>
       </c>
       <c r="D610">
         <v>14.98</v>
@@ -8967,10 +8967,10 @@
         <v>2023-11</v>
       </c>
       <c r="B611">
-        <v>50.6</v>
+        <v>50.62</v>
       </c>
       <c r="C611">
-        <v>42.59</v>
+        <v>42.57</v>
       </c>
       <c r="D611">
         <v>14.78</v>
@@ -8985,7 +8985,7 @@
         <v>44.92</v>
       </c>
       <c r="J611">
-        <v>-9.02</v>
+        <v>-9.01</v>
       </c>
     </row>
     <row r="612">
@@ -8993,10 +8993,10 @@
         <v>2023-12</v>
       </c>
       <c r="B612">
-        <v>51.31</v>
+        <v>51.32</v>
       </c>
       <c r="C612">
-        <v>43.64</v>
+        <v>43.61</v>
       </c>
       <c r="D612">
         <v>15.14</v>
@@ -9011,7 +9011,7 @@
         <v>44.18</v>
       </c>
       <c r="J612">
-        <v>-9.84</v>
+        <v>-9.83</v>
       </c>
     </row>
     <row r="613">
@@ -9019,10 +9019,10 @@
         <v>2024-01</v>
       </c>
       <c r="B613">
-        <v>51.52</v>
+        <v>51.54</v>
       </c>
       <c r="C613">
-        <v>42.63</v>
+        <v>42.6</v>
       </c>
       <c r="D613">
         <v>13.43</v>
@@ -9043,7 +9043,7 @@
         <v>7.6</v>
       </c>
       <c r="J613">
-        <v>-13.78</v>
+        <v>-13.77</v>
       </c>
     </row>
     <row r="614">
@@ -9051,10 +9051,10 @@
         <v>2024-02</v>
       </c>
       <c r="B614">
-        <v>52.6</v>
+        <v>52.62</v>
       </c>
       <c r="C614">
-        <v>39.52</v>
+        <v>39.47</v>
       </c>
       <c r="D614">
         <v>13.04</v>
@@ -9069,7 +9069,7 @@
         <v>48.79</v>
       </c>
       <c r="J614">
-        <v>-15.84</v>
+        <v>-15.82</v>
       </c>
     </row>
     <row r="615">
@@ -9077,10 +9077,10 @@
         <v>2024-03</v>
       </c>
       <c r="B615">
-        <v>51.25</v>
+        <v>51.16</v>
       </c>
       <c r="C615">
-        <v>39.66</v>
+        <v>39.62</v>
       </c>
       <c r="D615">
         <v>13.27</v>
@@ -9095,7 +9095,7 @@
         <v>43.69</v>
       </c>
       <c r="J615">
-        <v>-15.87</v>
+        <v>-15.86</v>
       </c>
     </row>
     <row r="616">
@@ -9103,10 +9103,10 @@
         <v>2024-04</v>
       </c>
       <c r="B616">
-        <v>49.68</v>
+        <v>49.67</v>
       </c>
       <c r="C616">
-        <v>39.04</v>
+        <v>39.19</v>
       </c>
       <c r="D616">
         <v>13.08</v>
@@ -9127,7 +9127,7 @@
         <v>-1.98</v>
       </c>
       <c r="J616">
-        <v>-12.92</v>
+        <v>-12.93</v>
       </c>
     </row>
     <row r="617">
@@ -9138,7 +9138,7 @@
         <v>51.12</v>
       </c>
       <c r="C617">
-        <v>37.29</v>
+        <v>37.31</v>
       </c>
       <c r="D617">
         <v>13.47</v>
@@ -9153,7 +9153,7 @@
         <v>51.07</v>
       </c>
       <c r="J617">
-        <v>-13.01</v>
+        <v>-13.02</v>
       </c>
     </row>
     <row r="618">
@@ -9164,7 +9164,7 @@
         <v>49.31</v>
       </c>
       <c r="C618">
-        <v>37.06</v>
+        <v>37.07</v>
       </c>
       <c r="D618">
         <v>10.48</v>
@@ -9190,7 +9190,7 @@
         <v>51.16</v>
       </c>
       <c r="C619">
-        <v>33.09</v>
+        <v>33.1</v>
       </c>
       <c r="D619">
         <v>11.27</v>
@@ -9211,7 +9211,7 @@
         <v>-7.1</v>
       </c>
       <c r="J619">
-        <v>-8.09</v>
+        <v>-8.1</v>
       </c>
     </row>
     <row r="620">
@@ -9237,7 +9237,7 @@
         <v>48.22</v>
       </c>
       <c r="J620">
-        <v>-4.99</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="621">
@@ -9248,7 +9248,7 @@
         <v>53.1</v>
       </c>
       <c r="C621">
-        <v>36.52</v>
+        <v>36.51</v>
       </c>
       <c r="D621">
         <v>12.58</v>
@@ -9271,10 +9271,10 @@
         <v>2024-10</v>
       </c>
       <c r="B622">
-        <v>49.97</v>
+        <v>50.03</v>
       </c>
       <c r="C622">
-        <v>36.69</v>
+        <v>36.67</v>
       </c>
       <c r="D622">
         <v>13.32</v>
@@ -9303,10 +9303,10 @@
         <v>2024-11</v>
       </c>
       <c r="B623">
-        <v>52.62</v>
+        <v>52.64</v>
       </c>
       <c r="C623">
-        <v>40.24</v>
+        <v>40.22</v>
       </c>
       <c r="D623">
         <v>13.24</v>
@@ -9329,10 +9329,10 @@
         <v>2024-12</v>
       </c>
       <c r="B624">
-        <v>52.89</v>
+        <v>52.91</v>
       </c>
       <c r="C624">
-        <v>36.05</v>
+        <v>36.01</v>
       </c>
       <c r="D624">
         <v>13.29</v>
@@ -9347,7 +9347,7 @@
         <v>50.25</v>
       </c>
       <c r="J624">
-        <v>-7.43</v>
+        <v>-7.41</v>
       </c>
     </row>
     <row r="625">
@@ -9355,10 +9355,10 @@
         <v>2025-01</v>
       </c>
       <c r="B625">
-        <v>51.66</v>
+        <v>51.68</v>
       </c>
       <c r="C625">
-        <v>35.36</v>
+        <v>35.32</v>
       </c>
       <c r="D625">
         <v>11.94</v>
@@ -9379,7 +9379,7 @@
         <v>-1.65</v>
       </c>
       <c r="J625">
-        <v>-11.33</v>
+        <v>-11.32</v>
       </c>
     </row>
     <row r="626">
@@ -9387,10 +9387,10 @@
         <v>2025-02</v>
       </c>
       <c r="B626">
-        <v>50.18</v>
+        <v>50.21</v>
       </c>
       <c r="C626">
-        <v>38.22</v>
+        <v>38.16</v>
       </c>
       <c r="D626">
         <v>11.41</v>
@@ -9405,7 +9405,7 @@
         <v>38.09</v>
       </c>
       <c r="J626">
-        <v>-11.83</v>
+        <v>-11.81</v>
       </c>
     </row>
     <row r="627">
@@ -9413,10 +9413,10 @@
         <v>2025-03</v>
       </c>
       <c r="B627">
-        <v>51.75</v>
+        <v>51.61</v>
       </c>
       <c r="C627">
-        <v>35.48</v>
+        <v>35.42</v>
       </c>
       <c r="D627">
         <v>10.85</v>
@@ -9431,7 +9431,7 @@
         <v>37.2</v>
       </c>
       <c r="J627">
-        <v>-11.78</v>
+        <v>-11.77</v>
       </c>
     </row>
     <row r="628">
@@ -9439,10 +9439,10 @@
         <v>2025-04</v>
       </c>
       <c r="B628">
-        <v>48.56</v>
+        <v>48.54</v>
       </c>
       <c r="C628">
-        <v>33.97</v>
+        <v>34.17</v>
       </c>
       <c r="D628">
         <v>9.26</v>
@@ -9463,7 +9463,7 @@
         <v>-2.37</v>
       </c>
       <c r="J628">
-        <v>-12.03</v>
+        <v>-12.04</v>
       </c>
     </row>
     <row r="629">
@@ -9474,7 +9474,7 @@
         <v>49.07</v>
       </c>
       <c r="C629">
-        <v>38.54</v>
+        <v>38.57</v>
       </c>
       <c r="D629">
         <v>10.3</v>
@@ -9489,7 +9489,7 @@
         <v>32.29</v>
       </c>
       <c r="J629">
-        <v>-9.31</v>
+        <v>-9.33</v>
       </c>
     </row>
     <row r="630">
@@ -9500,7 +9500,7 @@
         <v>51.27</v>
       </c>
       <c r="C630">
-        <v>38.37</v>
+        <v>38.38</v>
       </c>
       <c r="D630">
         <v>11.26</v>
@@ -9526,7 +9526,7 @@
         <v>50.52</v>
       </c>
       <c r="C631">
-        <v>37.2</v>
+        <v>37.21</v>
       </c>
       <c r="D631">
         <v>11.95</v>
@@ -9547,7 +9547,7 @@
         <v>0.27</v>
       </c>
       <c r="J631">
-        <v>-7.52</v>
+        <v>-7.54</v>
       </c>
     </row>
     <row r="632">
@@ -9558,7 +9558,7 @@
         <v>47.77</v>
       </c>
       <c r="C632">
-        <v>37.15</v>
+        <v>37.16</v>
       </c>
       <c r="D632">
         <v>9.19</v>
@@ -9573,7 +9573,7 @@
         <v>36.16</v>
       </c>
       <c r="J632">
-        <v>-17.84</v>
+        <v>-17.85</v>
       </c>
     </row>
     <row r="633">
@@ -9581,7 +9581,7 @@
         <v>2025-09</v>
       </c>
       <c r="B633">
-        <v>48.02</v>
+        <v>48.03</v>
       </c>
       <c r="C633">
         <v>39.38</v>
@@ -9607,10 +9607,10 @@
         <v>2025-10</v>
       </c>
       <c r="B634">
-        <v>52.42</v>
+        <v>52.49</v>
       </c>
       <c r="C634">
-        <v>34.69</v>
+        <v>34.67</v>
       </c>
       <c r="D634">
         <v>12.67</v>
@@ -9639,10 +9639,10 @@
         <v>2025-11</v>
       </c>
       <c r="B635">
-        <v>50.29</v>
+        <v>50.32</v>
       </c>
       <c r="C635">
-        <v>38.78</v>
+        <v>38.76</v>
       </c>
       <c r="D635">
         <v>12.51</v>
@@ -9657,7 +9657,7 @@
         <v>38.73</v>
       </c>
       <c r="J635">
-        <v>-10.15</v>
+        <v>-10.14</v>
       </c>
     </row>
     <row r="636">
@@ -9665,10 +9665,10 @@
         <v>2025-12</v>
       </c>
       <c r="B636">
-        <v>47.66</v>
+        <v>47.68</v>
       </c>
       <c r="C636">
-        <v>39.54</v>
+        <v>39.5</v>
       </c>
       <c r="D636">
         <v>12.87</v>
@@ -9683,7 +9683,7 @@
         <v>39.09</v>
       </c>
       <c r="J636">
-        <v>-7.3</v>
+        <v>-7.28</v>
       </c>
     </row>
     <row r="637">
@@ -9691,10 +9691,10 @@
         <v>2026-01</v>
       </c>
       <c r="B637">
-        <v>47.59</v>
+        <v>47.62</v>
       </c>
       <c r="C637">
-        <v>40.72</v>
+        <v>40.66</v>
       </c>
       <c r="D637">
         <v>17.61</v>
@@ -9715,7 +9715,7 @@
         <v>6.41</v>
       </c>
       <c r="J637">
-        <v>7.2</v>
+        <v>7.22</v>
       </c>
     </row>
     <row r="638">
@@ -9723,10 +9723,10 @@
         <v>2026-02</v>
       </c>
       <c r="B638">
-        <v>47.69</v>
+        <v>47.72</v>
       </c>
       <c r="C638">
-        <v>43.78</v>
+        <v>43.7</v>
       </c>
       <c r="D638">
         <v>17.58</v>
@@ -9741,7 +9741,7 @@
         <v>43.85</v>
       </c>
       <c r="J638">
-        <v>3.96</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="639">
@@ -9749,10 +9749,10 @@
         <v>2026-03</v>
       </c>
       <c r="B639">
-        <v>46.84</v>
+        <v>46.67</v>
       </c>
       <c r="C639">
-        <v>45.61</v>
+        <v>45.54</v>
       </c>
       <c r="D639">
         <v>16.56</v>
@@ -9767,7 +9767,7 @@
         <v>43.39</v>
       </c>
       <c r="J639">
-        <v>-0.57</v>
+        <v>-0.56</v>
       </c>
     </row>
     <row r="640">
@@ -9775,10 +9775,10 @@
         <v>2026-04</v>
       </c>
       <c r="B640">
-        <v>52.42</v>
+        <v>52.64</v>
       </c>
       <c r="C640">
-        <v>45.14</v>
+        <v>44.82</v>
       </c>
       <c r="D640">
         <v>18.25</v>
@@ -9799,7 +9799,7 @@
         <v>8.79</v>
       </c>
       <c r="J640">
-        <v>4.12</v>
+        <v>4.36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add commodities report and inputs related to commodities marekt
</commit_message>
<xml_diff>
--- a/data/excel/kof_indicator_business_situation.xlsx
+++ b/data/excel/kof_indicator_business_situation.xlsx
@@ -7603,7 +7603,7 @@
         <v>-1.64</v>
       </c>
       <c r="F562">
-        <v>24.07</v>
+        <v>24.18</v>
       </c>
       <c r="G562">
         <v>41.89</v>
@@ -7635,7 +7635,7 @@
         <v>2.09</v>
       </c>
       <c r="F563">
-        <v>23.69</v>
+        <v>23.7</v>
       </c>
       <c r="G563">
         <v>43.1</v>
@@ -7687,7 +7687,7 @@
         <v>3.26</v>
       </c>
       <c r="F565">
-        <v>28</v>
+        <v>27.99</v>
       </c>
       <c r="G565">
         <v>40.07</v>
@@ -7745,7 +7745,7 @@
         <v>1.28</v>
       </c>
       <c r="F567">
-        <v>18.39</v>
+        <v>18.31</v>
       </c>
       <c r="G567">
         <v>31.24</v>
@@ -7771,7 +7771,7 @@
         <v>-23.3</v>
       </c>
       <c r="F568">
-        <v>-32.27</v>
+        <v>-32.25</v>
       </c>
       <c r="G568">
         <v>10.7</v>
@@ -7803,7 +7803,7 @@
         <v>-25.4</v>
       </c>
       <c r="F569">
-        <v>-40.56</v>
+        <v>-40.7</v>
       </c>
       <c r="G569">
         <v>26.29</v>
@@ -7829,7 +7829,7 @@
         <v>-7.25</v>
       </c>
       <c r="F570">
-        <v>-29.73</v>
+        <v>-29.7</v>
       </c>
       <c r="G570">
         <v>24.37</v>
@@ -7855,7 +7855,7 @@
         <v>5.14</v>
       </c>
       <c r="F571">
-        <v>-18.54</v>
+        <v>-18.56</v>
       </c>
       <c r="G571">
         <v>27.5</v>
@@ -7887,7 +7887,7 @@
         <v>9.5</v>
       </c>
       <c r="F572">
-        <v>-18.35</v>
+        <v>-18.31</v>
       </c>
       <c r="G572">
         <v>26.95</v>
@@ -7913,7 +7913,7 @@
         <v>11.22</v>
       </c>
       <c r="F573">
-        <v>-7.34</v>
+        <v>-7.32</v>
       </c>
       <c r="G573">
         <v>25.18</v>
@@ -7939,7 +7939,7 @@
         <v>8.67</v>
       </c>
       <c r="F574">
-        <v>-1.68</v>
+        <v>-1.56</v>
       </c>
       <c r="G574">
         <v>35.42</v>
@@ -7997,7 +7997,7 @@
         <v>-0.61</v>
       </c>
       <c r="F576">
-        <v>-5.72</v>
+        <v>-5.73</v>
       </c>
       <c r="G576">
         <v>34.87</v>
@@ -8023,7 +8023,7 @@
         <v>0.04</v>
       </c>
       <c r="F577">
-        <v>-6.42</v>
+        <v>-6.43</v>
       </c>
       <c r="G577">
         <v>33.2</v>
@@ -8081,10 +8081,10 @@
         <v>-8.84</v>
       </c>
       <c r="F579">
-        <v>-6.02</v>
+        <v>-6.09</v>
       </c>
       <c r="G579">
-        <v>39.88</v>
+        <v>39.89</v>
       </c>
       <c r="J579">
         <v>4.33</v>
@@ -8107,7 +8107,7 @@
         <v>6.79</v>
       </c>
       <c r="F580">
-        <v>-1.42</v>
+        <v>-1.4</v>
       </c>
       <c r="G580">
         <v>34.66</v>
@@ -8139,7 +8139,7 @@
         <v>12.78</v>
       </c>
       <c r="F581">
-        <v>-0.04</v>
+        <v>-0.14</v>
       </c>
       <c r="G581">
         <v>39.8</v>
@@ -8165,7 +8165,7 @@
         <v>14.26</v>
       </c>
       <c r="F582">
-        <v>4.3</v>
+        <v>4.33</v>
       </c>
       <c r="G582">
         <v>38.75</v>
@@ -8223,7 +8223,7 @@
         <v>13.71</v>
       </c>
       <c r="F584">
-        <v>9.81</v>
+        <v>9.84</v>
       </c>
       <c r="G584">
         <v>50.62</v>
@@ -8249,7 +8249,7 @@
         <v>11.98</v>
       </c>
       <c r="F585">
-        <v>14.17</v>
+        <v>14.16</v>
       </c>
       <c r="G585">
         <v>61.67</v>
@@ -8275,7 +8275,7 @@
         <v>12.03</v>
       </c>
       <c r="F586">
-        <v>16.09</v>
+        <v>16.21</v>
       </c>
       <c r="G586">
         <v>49.7</v>
@@ -8310,7 +8310,7 @@
         <v>16.93</v>
       </c>
       <c r="G587">
-        <v>44.84</v>
+        <v>44.85</v>
       </c>
       <c r="J587">
         <v>31.56</v>
@@ -8333,7 +8333,7 @@
         <v>15</v>
       </c>
       <c r="F588">
-        <v>16.76</v>
+        <v>16.75</v>
       </c>
       <c r="G588">
         <v>46.36</v>
@@ -8359,10 +8359,10 @@
         <v>12.45</v>
       </c>
       <c r="F589">
-        <v>15.32</v>
+        <v>15.31</v>
       </c>
       <c r="G589">
-        <v>47.04</v>
+        <v>47.05</v>
       </c>
       <c r="H589">
         <v>-24.94</v>
@@ -8394,7 +8394,7 @@
         <v>25.18</v>
       </c>
       <c r="G590">
-        <v>43.48</v>
+        <v>43.49</v>
       </c>
       <c r="J590">
         <v>31.41</v>
@@ -8417,10 +8417,10 @@
         <v>15.41</v>
       </c>
       <c r="F591">
-        <v>24.34</v>
+        <v>24.3</v>
       </c>
       <c r="G591">
-        <v>30.9</v>
+        <v>30.91</v>
       </c>
       <c r="J591">
         <v>30.81</v>
@@ -8443,10 +8443,10 @@
         <v>12.23</v>
       </c>
       <c r="F592">
-        <v>25.9</v>
+        <v>25.91</v>
       </c>
       <c r="G592">
-        <v>39.01</v>
+        <v>39</v>
       </c>
       <c r="H592">
         <v>5.67</v>
@@ -8475,7 +8475,7 @@
         <v>12.38</v>
       </c>
       <c r="F593">
-        <v>26.01</v>
+        <v>25.95</v>
       </c>
       <c r="G593">
         <v>38.52</v>
@@ -8501,7 +8501,7 @@
         <v>12.29</v>
       </c>
       <c r="F594">
-        <v>23.62</v>
+        <v>23.64</v>
       </c>
       <c r="G594">
         <v>36.87</v>
@@ -8530,7 +8530,7 @@
         <v>22.82</v>
       </c>
       <c r="G595">
-        <v>28.49</v>
+        <v>28.48</v>
       </c>
       <c r="H595">
         <v>27.36</v>
@@ -8559,10 +8559,10 @@
         <v>5.28</v>
       </c>
       <c r="F596">
-        <v>21.57</v>
+        <v>21.58</v>
       </c>
       <c r="G596">
-        <v>26.96</v>
+        <v>26.95</v>
       </c>
       <c r="J596">
         <v>23.02</v>
@@ -8585,7 +8585,7 @@
         <v>6.9</v>
       </c>
       <c r="F597">
-        <v>20.06</v>
+        <v>20.02</v>
       </c>
       <c r="G597">
         <v>30.97</v>
@@ -8611,7 +8611,7 @@
         <v>9.48</v>
       </c>
       <c r="F598">
-        <v>16.69</v>
+        <v>16.82</v>
       </c>
       <c r="G598">
         <v>23.87</v>
@@ -8643,7 +8643,7 @@
         <v>8.47</v>
       </c>
       <c r="F599">
-        <v>18.47</v>
+        <v>18.45</v>
       </c>
       <c r="G599">
         <v>27.25</v>
@@ -8669,7 +8669,7 @@
         <v>14.45</v>
       </c>
       <c r="F600">
-        <v>18.79</v>
+        <v>18.78</v>
       </c>
       <c r="G600">
         <v>27.85</v>
@@ -8695,10 +8695,10 @@
         <v>13.79</v>
       </c>
       <c r="F601">
-        <v>20.39</v>
+        <v>20.37</v>
       </c>
       <c r="G601">
-        <v>35.26</v>
+        <v>35.27</v>
       </c>
       <c r="H601">
         <v>27.98</v>
@@ -8727,10 +8727,10 @@
         <v>12.98</v>
       </c>
       <c r="F602">
-        <v>21.76</v>
+        <v>21.75</v>
       </c>
       <c r="G602">
-        <v>36.74</v>
+        <v>36.76</v>
       </c>
       <c r="J602">
         <v>18.74</v>
@@ -8753,10 +8753,10 @@
         <v>12.75</v>
       </c>
       <c r="F603">
-        <v>21.46</v>
+        <v>21.44</v>
       </c>
       <c r="G603">
-        <v>43.95</v>
+        <v>43.97</v>
       </c>
       <c r="J603">
         <v>16.94</v>
@@ -8779,10 +8779,10 @@
         <v>11.56</v>
       </c>
       <c r="F604">
-        <v>18.99</v>
+        <v>19.01</v>
       </c>
       <c r="G604">
-        <v>44.31</v>
+        <v>44.3</v>
       </c>
       <c r="H604">
         <v>26.87</v>
@@ -8811,10 +8811,10 @@
         <v>5.83</v>
       </c>
       <c r="F605">
-        <v>22.28</v>
+        <v>22.26</v>
       </c>
       <c r="G605">
-        <v>42.49</v>
+        <v>42.47</v>
       </c>
       <c r="J605">
         <v>-0.15</v>
@@ -8837,10 +8837,10 @@
         <v>5.86</v>
       </c>
       <c r="F606">
-        <v>18.47</v>
+        <v>18.5</v>
       </c>
       <c r="G606">
-        <v>42.27</v>
+        <v>42.26</v>
       </c>
       <c r="J606">
         <v>-0.55</v>
@@ -8863,7 +8863,7 @@
         <v>8.37</v>
       </c>
       <c r="F607">
-        <v>16.62</v>
+        <v>16.63</v>
       </c>
       <c r="G607">
         <v>44.74</v>
@@ -8921,7 +8921,7 @@
         <v>7.66</v>
       </c>
       <c r="F609">
-        <v>14.07</v>
+        <v>14.01</v>
       </c>
       <c r="G609">
         <v>41.5</v>
@@ -8947,7 +8947,7 @@
         <v>4.35</v>
       </c>
       <c r="F610">
-        <v>14.22</v>
+        <v>14.31</v>
       </c>
       <c r="G610">
         <v>49.82</v>
@@ -8979,10 +8979,10 @@
         <v>5.39</v>
       </c>
       <c r="F611">
-        <v>14.94</v>
+        <v>14.93</v>
       </c>
       <c r="G611">
-        <v>44.92</v>
+        <v>44.93</v>
       </c>
       <c r="J611">
         <v>-9.01</v>
@@ -9005,10 +9005,10 @@
         <v>2.8</v>
       </c>
       <c r="F612">
-        <v>16.72</v>
+        <v>16.7</v>
       </c>
       <c r="G612">
-        <v>44.18</v>
+        <v>44.19</v>
       </c>
       <c r="J612">
         <v>-9.83</v>
@@ -9031,10 +9031,10 @@
         <v>3.82</v>
       </c>
       <c r="F613">
-        <v>17.24</v>
+        <v>17.21</v>
       </c>
       <c r="G613">
-        <v>44.53</v>
+        <v>44.55</v>
       </c>
       <c r="H613">
         <v>12</v>
@@ -9063,10 +9063,10 @@
         <v>3.87</v>
       </c>
       <c r="F614">
-        <v>16.69</v>
+        <v>16.67</v>
       </c>
       <c r="G614">
-        <v>48.79</v>
+        <v>48.82</v>
       </c>
       <c r="J614">
         <v>-15.82</v>
@@ -9089,10 +9089,10 @@
         <v>6.77</v>
       </c>
       <c r="F615">
-        <v>18.55</v>
+        <v>18.53</v>
       </c>
       <c r="G615">
-        <v>43.69</v>
+        <v>43.72</v>
       </c>
       <c r="J615">
         <v>-15.86</v>
@@ -9115,10 +9115,10 @@
         <v>3.48</v>
       </c>
       <c r="F616">
-        <v>19.35</v>
+        <v>19.39</v>
       </c>
       <c r="G616">
-        <v>46.8</v>
+        <v>46.76</v>
       </c>
       <c r="H616">
         <v>5.23</v>
@@ -9147,10 +9147,10 @@
         <v>1.71</v>
       </c>
       <c r="F617">
-        <v>19.54</v>
+        <v>19.56</v>
       </c>
       <c r="G617">
-        <v>51.07</v>
+        <v>51.03</v>
       </c>
       <c r="J617">
         <v>-13.02</v>
@@ -9173,10 +9173,10 @@
         <v>0.32</v>
       </c>
       <c r="F618">
-        <v>18.9</v>
+        <v>18.94</v>
       </c>
       <c r="G618">
-        <v>47.74</v>
+        <v>47.72</v>
       </c>
       <c r="J618">
         <v>-22.46</v>
@@ -9202,7 +9202,7 @@
         <v>15.22</v>
       </c>
       <c r="G619">
-        <v>46.77</v>
+        <v>46.76</v>
       </c>
       <c r="H619">
         <v>2.36</v>
@@ -9231,7 +9231,7 @@
         <v>-0.33</v>
       </c>
       <c r="F620">
-        <v>15.06</v>
+        <v>15.05</v>
       </c>
       <c r="G620">
         <v>48.22</v>
@@ -9257,7 +9257,7 @@
         <v>-2.02</v>
       </c>
       <c r="F621">
-        <v>18.59</v>
+        <v>18.57</v>
       </c>
       <c r="G621">
         <v>47.73</v>
@@ -9283,7 +9283,7 @@
         <v>-2.33</v>
       </c>
       <c r="F622">
-        <v>19.61</v>
+        <v>19.67</v>
       </c>
       <c r="G622">
         <v>43.92</v>
@@ -9315,10 +9315,10 @@
         <v>-0.97</v>
       </c>
       <c r="F623">
-        <v>16.84</v>
+        <v>16.82</v>
       </c>
       <c r="G623">
-        <v>45.55</v>
+        <v>45.56</v>
       </c>
       <c r="J623">
         <v>-6.53</v>
@@ -9341,10 +9341,10 @@
         <v>-0.7</v>
       </c>
       <c r="F624">
-        <v>16.71</v>
+        <v>16.69</v>
       </c>
       <c r="G624">
-        <v>50.25</v>
+        <v>50.26</v>
       </c>
       <c r="J624">
         <v>-7.41</v>
@@ -9367,10 +9367,10 @@
         <v>-0.2</v>
       </c>
       <c r="F625">
-        <v>16.84</v>
+        <v>16.81</v>
       </c>
       <c r="G625">
-        <v>42.36</v>
+        <v>42.39</v>
       </c>
       <c r="H625">
         <v>3.28</v>
@@ -9399,10 +9399,10 @@
         <v>-1.43</v>
       </c>
       <c r="F626">
-        <v>16.79</v>
+        <v>16.75</v>
       </c>
       <c r="G626">
-        <v>38.09</v>
+        <v>38.13</v>
       </c>
       <c r="J626">
         <v>-11.81</v>
@@ -9425,10 +9425,10 @@
         <v>0.92</v>
       </c>
       <c r="F627">
-        <v>15.65</v>
+        <v>15.59</v>
       </c>
       <c r="G627">
-        <v>37.2</v>
+        <v>37.25</v>
       </c>
       <c r="J627">
         <v>-11.77</v>
@@ -9451,10 +9451,10 @@
         <v>-0.38</v>
       </c>
       <c r="F628">
-        <v>13.46</v>
+        <v>13.55</v>
       </c>
       <c r="G628">
-        <v>33.99</v>
+        <v>33.92</v>
       </c>
       <c r="H628">
         <v>3</v>
@@ -9483,10 +9483,10 @@
         <v>8.58</v>
       </c>
       <c r="F629">
-        <v>13.45</v>
+        <v>13.49</v>
       </c>
       <c r="G629">
-        <v>32.29</v>
+        <v>32.24</v>
       </c>
       <c r="J629">
         <v>-9.33</v>
@@ -9509,10 +9509,10 @@
         <v>2.8</v>
       </c>
       <c r="F630">
-        <v>13.62</v>
+        <v>13.67</v>
       </c>
       <c r="G630">
-        <v>38.29</v>
+        <v>38.27</v>
       </c>
       <c r="J630">
         <v>-7.39</v>
@@ -9538,7 +9538,7 @@
         <v>14.88</v>
       </c>
       <c r="G631">
-        <v>37.69</v>
+        <v>37.68</v>
       </c>
       <c r="H631">
         <v>5.21</v>
@@ -9567,7 +9567,7 @@
         <v>1.21</v>
       </c>
       <c r="F632">
-        <v>14.32</v>
+        <v>14.3</v>
       </c>
       <c r="G632">
         <v>36.16</v>
@@ -9596,7 +9596,7 @@
         <v>15.53</v>
       </c>
       <c r="G633">
-        <v>37.27</v>
+        <v>37.28</v>
       </c>
       <c r="J633">
         <v>-17.86</v>
@@ -9619,10 +9619,10 @@
         <v>2.65</v>
       </c>
       <c r="F634">
-        <v>16.19</v>
+        <v>16.22</v>
       </c>
       <c r="G634">
-        <v>36.15</v>
+        <v>36.16</v>
       </c>
       <c r="H634">
         <v>5.95</v>
@@ -9651,10 +9651,10 @@
         <v>2.17</v>
       </c>
       <c r="F635">
-        <v>18.15</v>
+        <v>18.13</v>
       </c>
       <c r="G635">
-        <v>38.73</v>
+        <v>38.75</v>
       </c>
       <c r="J635">
         <v>-10.14</v>
@@ -9677,10 +9677,10 @@
         <v>2.59</v>
       </c>
       <c r="F636">
-        <v>17.28</v>
+        <v>17.26</v>
       </c>
       <c r="G636">
-        <v>39.09</v>
+        <v>39.11</v>
       </c>
       <c r="J636">
         <v>-7.28</v>
@@ -9703,10 +9703,10 @@
         <v>3.38</v>
       </c>
       <c r="F637">
-        <v>17.82</v>
+        <v>17.78</v>
       </c>
       <c r="G637">
-        <v>42.23</v>
+        <v>42.26</v>
       </c>
       <c r="H637">
         <v>8.2</v>
@@ -9735,10 +9735,10 @@
         <v>4.68</v>
       </c>
       <c r="F638">
-        <v>18.71</v>
+        <v>18.65</v>
       </c>
       <c r="G638">
-        <v>43.85</v>
+        <v>43.9</v>
       </c>
       <c r="J638">
         <v>3.99</v>
@@ -9761,10 +9761,10 @@
         <v>2.08</v>
       </c>
       <c r="F639">
-        <v>19.01</v>
+        <v>18.9</v>
       </c>
       <c r="G639">
-        <v>43.39</v>
+        <v>43.44</v>
       </c>
       <c r="J639">
         <v>-0.56</v>
@@ -9787,10 +9787,10 @@
         <v>2.53</v>
       </c>
       <c r="F640">
-        <v>19.9</v>
+        <v>19.44</v>
       </c>
       <c r="G640">
-        <v>42.23</v>
+        <v>42.6</v>
       </c>
       <c r="H640">
         <v>4.75</v>

</xml_diff>

<commit_message>
add commodities energy, hard and soft reports and change publish scripts
</commit_message>
<xml_diff>
--- a/data/excel/kof_indicator_business_situation.xlsx
+++ b/data/excel/kof_indicator_business_situation.xlsx
@@ -7320,7 +7320,7 @@
         <v>28.46</v>
       </c>
       <c r="E551">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="G551">
         <v>39.34</v>
@@ -7597,7 +7597,7 @@
         <v>29.32</v>
       </c>
       <c r="D562">
-        <v>20.49</v>
+        <v>20.52</v>
       </c>
       <c r="E562">
         <v>-1.64</v>
@@ -7739,7 +7739,7 @@
         <v>32.59</v>
       </c>
       <c r="D567">
-        <v>15.85</v>
+        <v>15.82</v>
       </c>
       <c r="E567">
         <v>1.28</v>
@@ -7797,7 +7797,7 @@
         <v>1.16</v>
       </c>
       <c r="D569">
-        <v>-20.91</v>
+        <v>-20.95</v>
       </c>
       <c r="E569">
         <v>-25.4</v>
@@ -7823,7 +7823,7 @@
         <v>3.25</v>
       </c>
       <c r="D570">
-        <v>-17.44</v>
+        <v>-17.43</v>
       </c>
       <c r="E570">
         <v>-7.25</v>
@@ -7881,7 +7881,7 @@
         <v>16.21</v>
       </c>
       <c r="D572">
-        <v>-8.15</v>
+        <v>-8.13</v>
       </c>
       <c r="E572">
         <v>9.5</v>
@@ -7907,7 +7907,7 @@
         <v>16.38</v>
       </c>
       <c r="D573">
-        <v>-4.49</v>
+        <v>-4.48</v>
       </c>
       <c r="E573">
         <v>11.22</v>
@@ -7933,7 +7933,7 @@
         <v>20.28</v>
       </c>
       <c r="D574">
-        <v>4.13</v>
+        <v>4.18</v>
       </c>
       <c r="E574">
         <v>8.67</v>
@@ -7991,7 +7991,7 @@
         <v>21.36</v>
       </c>
       <c r="D576">
-        <v>2.77</v>
+        <v>2.76</v>
       </c>
       <c r="E576">
         <v>-0.61</v>
@@ -8075,7 +8075,7 @@
         <v>28.89</v>
       </c>
       <c r="D579">
-        <v>3.7</v>
+        <v>3.67</v>
       </c>
       <c r="E579">
         <v>-8.84</v>
@@ -8101,7 +8101,7 @@
         <v>31.83</v>
       </c>
       <c r="D580">
-        <v>12.69</v>
+        <v>12.7</v>
       </c>
       <c r="E580">
         <v>6.79</v>
@@ -8133,7 +8133,7 @@
         <v>34.58</v>
       </c>
       <c r="D581">
-        <v>15.13</v>
+        <v>15.09</v>
       </c>
       <c r="E581">
         <v>12.78</v>
@@ -8159,7 +8159,7 @@
         <v>33.49</v>
       </c>
       <c r="D582">
-        <v>16.86</v>
+        <v>16.87</v>
       </c>
       <c r="E582">
         <v>14.26</v>
@@ -8188,7 +8188,7 @@
         <v>25.21</v>
       </c>
       <c r="E583">
-        <v>20.95</v>
+        <v>20.96</v>
       </c>
       <c r="F583">
         <v>8.17</v>
@@ -8217,7 +8217,7 @@
         <v>39.81</v>
       </c>
       <c r="D584">
-        <v>25.93</v>
+        <v>25.95</v>
       </c>
       <c r="E584">
         <v>13.71</v>
@@ -8243,7 +8243,7 @@
         <v>39.5</v>
       </c>
       <c r="D585">
-        <v>29.36</v>
+        <v>29.35</v>
       </c>
       <c r="E585">
         <v>11.98</v>
@@ -8269,7 +8269,7 @@
         <v>38.82</v>
       </c>
       <c r="D586">
-        <v>29.89</v>
+        <v>29.94</v>
       </c>
       <c r="E586">
         <v>12.03</v>
@@ -8304,7 +8304,7 @@
         <v>29.89</v>
       </c>
       <c r="E587">
-        <v>16.39</v>
+        <v>16.38</v>
       </c>
       <c r="F587">
         <v>16.93</v>
@@ -8327,10 +8327,10 @@
         <v>40.42</v>
       </c>
       <c r="D588">
-        <v>29.47</v>
+        <v>29.46</v>
       </c>
       <c r="E588">
-        <v>15</v>
+        <v>14.99</v>
       </c>
       <c r="F588">
         <v>16.75</v>
@@ -8388,7 +8388,7 @@
         <v>31.97</v>
       </c>
       <c r="E590">
-        <v>15.24</v>
+        <v>15.23</v>
       </c>
       <c r="F590">
         <v>25.18</v>
@@ -8411,7 +8411,7 @@
         <v>40.79</v>
       </c>
       <c r="D591">
-        <v>29.9</v>
+        <v>29.89</v>
       </c>
       <c r="E591">
         <v>15.41</v>
@@ -8469,7 +8469,7 @@
         <v>40.68</v>
       </c>
       <c r="D593">
-        <v>32.62</v>
+        <v>32.6</v>
       </c>
       <c r="E593">
         <v>12.38</v>
@@ -8495,7 +8495,7 @@
         <v>39.65</v>
       </c>
       <c r="D594">
-        <v>31.98</v>
+        <v>31.99</v>
       </c>
       <c r="E594">
         <v>12.29</v>
@@ -8556,7 +8556,7 @@
         <v>27.6</v>
       </c>
       <c r="E596">
-        <v>5.28</v>
+        <v>5.29</v>
       </c>
       <c r="F596">
         <v>21.58</v>
@@ -8579,10 +8579,10 @@
         <v>43.23</v>
       </c>
       <c r="D597">
-        <v>27.53</v>
+        <v>27.52</v>
       </c>
       <c r="E597">
-        <v>6.9</v>
+        <v>6.91</v>
       </c>
       <c r="F597">
         <v>20.02</v>
@@ -8605,7 +8605,7 @@
         <v>44.14</v>
       </c>
       <c r="D598">
-        <v>24.12</v>
+        <v>24.17</v>
       </c>
       <c r="E598">
         <v>9.48</v>
@@ -8637,7 +8637,7 @@
         <v>44.76</v>
       </c>
       <c r="D599">
-        <v>24.19</v>
+        <v>24.18</v>
       </c>
       <c r="E599">
         <v>8.47</v>
@@ -8663,7 +8663,7 @@
         <v>47.3</v>
       </c>
       <c r="D600">
-        <v>25.22</v>
+        <v>25.21</v>
       </c>
       <c r="E600">
         <v>14.45</v>
@@ -8689,10 +8689,10 @@
         <v>48.87</v>
       </c>
       <c r="D601">
-        <v>29.61</v>
+        <v>29.6</v>
       </c>
       <c r="E601">
-        <v>13.79</v>
+        <v>13.78</v>
       </c>
       <c r="F601">
         <v>20.37</v>
@@ -8724,7 +8724,7 @@
         <v>27.84</v>
       </c>
       <c r="E602">
-        <v>12.98</v>
+        <v>12.97</v>
       </c>
       <c r="F602">
         <v>21.75</v>
@@ -8750,7 +8750,7 @@
         <v>28.28</v>
       </c>
       <c r="E603">
-        <v>12.75</v>
+        <v>12.73</v>
       </c>
       <c r="F603">
         <v>21.44</v>
@@ -8773,10 +8773,10 @@
         <v>46.35</v>
       </c>
       <c r="D604">
-        <v>24.18</v>
+        <v>24.19</v>
       </c>
       <c r="E604">
-        <v>11.56</v>
+        <v>11.59</v>
       </c>
       <c r="F604">
         <v>19.01</v>
@@ -8805,10 +8805,10 @@
         <v>40.4</v>
       </c>
       <c r="D605">
-        <v>22.76</v>
+        <v>22.75</v>
       </c>
       <c r="E605">
-        <v>5.83</v>
+        <v>5.84</v>
       </c>
       <c r="F605">
         <v>22.26</v>
@@ -8831,10 +8831,10 @@
         <v>45.12</v>
       </c>
       <c r="D606">
-        <v>21.57</v>
+        <v>21.58</v>
       </c>
       <c r="E606">
-        <v>5.86</v>
+        <v>5.87</v>
       </c>
       <c r="F606">
         <v>18.5</v>
@@ -8860,7 +8860,7 @@
         <v>17.92</v>
       </c>
       <c r="E607">
-        <v>8.37</v>
+        <v>8.38</v>
       </c>
       <c r="F607">
         <v>16.63</v>
@@ -8915,7 +8915,7 @@
         <v>43.39</v>
       </c>
       <c r="D609">
-        <v>16.91</v>
+        <v>16.88</v>
       </c>
       <c r="E609">
         <v>7.66</v>
@@ -8941,7 +8941,7 @@
         <v>44.4</v>
       </c>
       <c r="D610">
-        <v>14.98</v>
+        <v>15.01</v>
       </c>
       <c r="E610">
         <v>4.35</v>
@@ -8976,7 +8976,7 @@
         <v>14.78</v>
       </c>
       <c r="E611">
-        <v>5.39</v>
+        <v>5.38</v>
       </c>
       <c r="F611">
         <v>14.93</v>
@@ -9002,7 +9002,7 @@
         <v>15.14</v>
       </c>
       <c r="E612">
-        <v>2.8</v>
+        <v>2.79</v>
       </c>
       <c r="F612">
         <v>16.7</v>
@@ -9025,10 +9025,10 @@
         <v>42.6</v>
       </c>
       <c r="D613">
-        <v>13.43</v>
+        <v>13.42</v>
       </c>
       <c r="E613">
-        <v>3.82</v>
+        <v>3.8</v>
       </c>
       <c r="F613">
         <v>17.21</v>
@@ -9060,7 +9060,7 @@
         <v>13.04</v>
       </c>
       <c r="E614">
-        <v>3.87</v>
+        <v>3.85</v>
       </c>
       <c r="F614">
         <v>16.67</v>
@@ -9083,10 +9083,10 @@
         <v>39.62</v>
       </c>
       <c r="D615">
-        <v>13.27</v>
+        <v>13.26</v>
       </c>
       <c r="E615">
-        <v>6.77</v>
+        <v>6.74</v>
       </c>
       <c r="F615">
         <v>18.53</v>
@@ -9109,10 +9109,10 @@
         <v>39.19</v>
       </c>
       <c r="D616">
-        <v>13.08</v>
+        <v>13.1</v>
       </c>
       <c r="E616">
-        <v>3.48</v>
+        <v>3.54</v>
       </c>
       <c r="F616">
         <v>19.39</v>
@@ -9144,7 +9144,7 @@
         <v>13.47</v>
       </c>
       <c r="E617">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="F617">
         <v>19.56</v>
@@ -9167,7 +9167,7 @@
         <v>37.07</v>
       </c>
       <c r="D618">
-        <v>10.48</v>
+        <v>10.49</v>
       </c>
       <c r="E618">
         <v>0.32</v>
@@ -9196,7 +9196,7 @@
         <v>11.27</v>
       </c>
       <c r="E619">
-        <v>-5.33</v>
+        <v>-5.31</v>
       </c>
       <c r="F619">
         <v>15.22</v>
@@ -9228,7 +9228,7 @@
         <v>12.63</v>
       </c>
       <c r="E620">
-        <v>-0.33</v>
+        <v>-0.32</v>
       </c>
       <c r="F620">
         <v>15.05</v>
@@ -9251,7 +9251,7 @@
         <v>36.51</v>
       </c>
       <c r="D621">
-        <v>12.58</v>
+        <v>12.57</v>
       </c>
       <c r="E621">
         <v>-2.02</v>
@@ -9277,7 +9277,7 @@
         <v>36.67</v>
       </c>
       <c r="D622">
-        <v>13.32</v>
+        <v>13.34</v>
       </c>
       <c r="E622">
         <v>-2.33</v>
@@ -9309,10 +9309,10 @@
         <v>40.22</v>
       </c>
       <c r="D623">
-        <v>13.24</v>
+        <v>13.23</v>
       </c>
       <c r="E623">
-        <v>-0.97</v>
+        <v>-0.99</v>
       </c>
       <c r="F623">
         <v>16.82</v>
@@ -9335,10 +9335,10 @@
         <v>36.01</v>
       </c>
       <c r="D624">
-        <v>13.29</v>
+        <v>13.28</v>
       </c>
       <c r="E624">
-        <v>-0.7</v>
+        <v>-0.72</v>
       </c>
       <c r="F624">
         <v>16.69</v>
@@ -9361,10 +9361,10 @@
         <v>35.32</v>
       </c>
       <c r="D625">
-        <v>11.94</v>
+        <v>11.93</v>
       </c>
       <c r="E625">
-        <v>-0.2</v>
+        <v>-0.22</v>
       </c>
       <c r="F625">
         <v>16.81</v>
@@ -9393,10 +9393,10 @@
         <v>38.16</v>
       </c>
       <c r="D626">
-        <v>11.41</v>
+        <v>11.4</v>
       </c>
       <c r="E626">
-        <v>-1.43</v>
+        <v>-1.46</v>
       </c>
       <c r="F626">
         <v>16.75</v>
@@ -9419,10 +9419,10 @@
         <v>35.42</v>
       </c>
       <c r="D627">
-        <v>10.85</v>
+        <v>10.83</v>
       </c>
       <c r="E627">
-        <v>0.92</v>
+        <v>0.88</v>
       </c>
       <c r="F627">
         <v>15.59</v>
@@ -9445,10 +9445,10 @@
         <v>34.17</v>
       </c>
       <c r="D628">
-        <v>9.26</v>
+        <v>9.3</v>
       </c>
       <c r="E628">
-        <v>-0.38</v>
+        <v>-0.27</v>
       </c>
       <c r="F628">
         <v>13.55</v>
@@ -9477,10 +9477,10 @@
         <v>38.57</v>
       </c>
       <c r="D629">
-        <v>10.3</v>
+        <v>10.31</v>
       </c>
       <c r="E629">
-        <v>8.58</v>
+        <v>8.59</v>
       </c>
       <c r="F629">
         <v>13.49</v>
@@ -9503,7 +9503,7 @@
         <v>38.38</v>
       </c>
       <c r="D630">
-        <v>11.26</v>
+        <v>11.28</v>
       </c>
       <c r="E630">
         <v>2.8</v>
@@ -9532,7 +9532,7 @@
         <v>11.95</v>
       </c>
       <c r="E631">
-        <v>2.09</v>
+        <v>2.12</v>
       </c>
       <c r="F631">
         <v>14.88</v>
@@ -9561,10 +9561,10 @@
         <v>37.16</v>
       </c>
       <c r="D632">
-        <v>9.19</v>
+        <v>9.18</v>
       </c>
       <c r="E632">
-        <v>1.21</v>
+        <v>1.22</v>
       </c>
       <c r="F632">
         <v>14.3</v>
@@ -9590,7 +9590,7 @@
         <v>9.94</v>
       </c>
       <c r="E633">
-        <v>1.76</v>
+        <v>1.75</v>
       </c>
       <c r="F633">
         <v>15.53</v>
@@ -9613,7 +9613,7 @@
         <v>34.67</v>
       </c>
       <c r="D634">
-        <v>12.67</v>
+        <v>12.68</v>
       </c>
       <c r="E634">
         <v>2.65</v>
@@ -9648,7 +9648,7 @@
         <v>12.51</v>
       </c>
       <c r="E635">
-        <v>2.17</v>
+        <v>2.15</v>
       </c>
       <c r="F635">
         <v>18.13</v>
@@ -9674,7 +9674,7 @@
         <v>12.87</v>
       </c>
       <c r="E636">
-        <v>2.59</v>
+        <v>2.57</v>
       </c>
       <c r="F636">
         <v>17.26</v>
@@ -9697,10 +9697,10 @@
         <v>40.66</v>
       </c>
       <c r="D637">
-        <v>17.61</v>
+        <v>17.6</v>
       </c>
       <c r="E637">
-        <v>3.38</v>
+        <v>3.35</v>
       </c>
       <c r="F637">
         <v>17.78</v>
@@ -9729,10 +9729,10 @@
         <v>43.7</v>
       </c>
       <c r="D638">
-        <v>17.58</v>
+        <v>17.57</v>
       </c>
       <c r="E638">
-        <v>4.68</v>
+        <v>4.64</v>
       </c>
       <c r="F638">
         <v>18.65</v>
@@ -9755,10 +9755,10 @@
         <v>45.54</v>
       </c>
       <c r="D639">
-        <v>16.56</v>
+        <v>16.52</v>
       </c>
       <c r="E639">
-        <v>2.08</v>
+        <v>2.03</v>
       </c>
       <c r="F639">
         <v>18.9</v>
@@ -9781,10 +9781,10 @@
         <v>44.82</v>
       </c>
       <c r="D640">
-        <v>18.25</v>
+        <v>18.13</v>
       </c>
       <c r="E640">
-        <v>2.53</v>
+        <v>1.99</v>
       </c>
       <c r="F640">
         <v>19.44</v>

</xml_diff>

<commit_message>
add gaz data and correct all html
</commit_message>
<xml_diff>
--- a/data/excel/kof_indicator_business_situation.xlsx
+++ b/data/excel/kof_indicator_business_situation.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J640"/>
+  <dimension ref="A1:J641"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5587,7 +5587,7 @@
         <v>8.57</v>
       </c>
       <c r="J484">
-        <v>-2.78</v>
+        <v>-2.79</v>
       </c>
     </row>
     <row r="485">
@@ -5789,7 +5789,7 @@
         <v>29.46</v>
       </c>
       <c r="J492">
-        <v>5.05</v>
+        <v>5.06</v>
       </c>
     </row>
     <row r="493">
@@ -6133,7 +6133,7 @@
         <v>23.13</v>
       </c>
       <c r="J505">
-        <v>9.75</v>
+        <v>9.76</v>
       </c>
     </row>
     <row r="506">
@@ -6156,7 +6156,7 @@
         <v>21.19</v>
       </c>
       <c r="J506">
-        <v>-8.86</v>
+        <v>-8.87</v>
       </c>
     </row>
     <row r="507">
@@ -6468,7 +6468,7 @@
         <v>17</v>
       </c>
       <c r="J518">
-        <v>-10.89</v>
+        <v>-10.9</v>
       </c>
     </row>
     <row r="519">
@@ -6523,7 +6523,7 @@
         <v>-8.06</v>
       </c>
       <c r="J520">
-        <v>-2.11</v>
+        <v>-2.12</v>
       </c>
     </row>
     <row r="521">
@@ -6679,7 +6679,7 @@
         <v>2.36</v>
       </c>
       <c r="J526">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="527">
@@ -6780,7 +6780,7 @@
         <v>30.64</v>
       </c>
       <c r="J530">
-        <v>-3.32</v>
+        <v>-3.33</v>
       </c>
     </row>
     <row r="531">
@@ -6803,7 +6803,7 @@
         <v>32.65</v>
       </c>
       <c r="J531">
-        <v>0.69</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="532">
@@ -6881,7 +6881,7 @@
         <v>37.93</v>
       </c>
       <c r="J534">
-        <v>9.93</v>
+        <v>9.94</v>
       </c>
     </row>
     <row r="535">
@@ -6959,7 +6959,7 @@
         <v>37.59</v>
       </c>
       <c r="J537">
-        <v>14.97</v>
+        <v>14.98</v>
       </c>
     </row>
     <row r="538">
@@ -6991,7 +6991,7 @@
         <v>18.18</v>
       </c>
       <c r="J538">
-        <v>17.61</v>
+        <v>17.62</v>
       </c>
     </row>
     <row r="539">
@@ -7092,7 +7092,7 @@
         <v>38.6</v>
       </c>
       <c r="J542">
-        <v>21.17</v>
+        <v>21.16</v>
       </c>
     </row>
     <row r="543">
@@ -7115,7 +7115,7 @@
         <v>43.02</v>
       </c>
       <c r="J543">
-        <v>21.98</v>
+        <v>21.95</v>
       </c>
     </row>
     <row r="544">
@@ -7147,7 +7147,7 @@
         <v>27.55</v>
       </c>
       <c r="J544">
-        <v>22.38</v>
+        <v>22.37</v>
       </c>
     </row>
     <row r="545">
@@ -7170,7 +7170,7 @@
         <v>44.47</v>
       </c>
       <c r="J545">
-        <v>27.12</v>
+        <v>27.13</v>
       </c>
     </row>
     <row r="546">
@@ -7193,7 +7193,7 @@
         <v>42</v>
       </c>
       <c r="J546">
-        <v>25.73</v>
+        <v>25.75</v>
       </c>
     </row>
     <row r="547">
@@ -7271,7 +7271,7 @@
         <v>40.79</v>
       </c>
       <c r="J549">
-        <v>26.3</v>
+        <v>26.31</v>
       </c>
     </row>
     <row r="550">
@@ -7303,7 +7303,7 @@
         <v>33.61</v>
       </c>
       <c r="J550">
-        <v>23.61</v>
+        <v>23.62</v>
       </c>
     </row>
     <row r="551">
@@ -7326,7 +7326,7 @@
         <v>39.34</v>
       </c>
       <c r="J551">
-        <v>26.78</v>
+        <v>26.79</v>
       </c>
     </row>
     <row r="552">
@@ -7349,7 +7349,7 @@
         <v>34.86</v>
       </c>
       <c r="J552">
-        <v>25.18</v>
+        <v>25.19</v>
       </c>
     </row>
     <row r="553">
@@ -7381,7 +7381,7 @@
         <v>27.12</v>
       </c>
       <c r="J553">
-        <v>21.76</v>
+        <v>21.77</v>
       </c>
     </row>
     <row r="554">
@@ -7427,7 +7427,7 @@
         <v>30.08</v>
       </c>
       <c r="J555">
-        <v>19.21</v>
+        <v>19.16</v>
       </c>
     </row>
     <row r="556">
@@ -7459,7 +7459,7 @@
         <v>26.34</v>
       </c>
       <c r="J556">
-        <v>15.29</v>
+        <v>15.27</v>
       </c>
     </row>
     <row r="557">
@@ -7482,7 +7482,7 @@
         <v>33.1</v>
       </c>
       <c r="J557">
-        <v>13.22</v>
+        <v>13.23</v>
       </c>
     </row>
     <row r="558">
@@ -7505,7 +7505,7 @@
         <v>33.47</v>
       </c>
       <c r="J558">
-        <v>11.63</v>
+        <v>11.66</v>
       </c>
     </row>
     <row r="559">
@@ -7537,7 +7537,7 @@
         <v>15.96</v>
       </c>
       <c r="J559">
-        <v>8.83</v>
+        <v>8.84</v>
       </c>
     </row>
     <row r="560">
@@ -7583,7 +7583,7 @@
         <v>38.89</v>
       </c>
       <c r="J561">
-        <v>5.94</v>
+        <v>5.95</v>
       </c>
     </row>
     <row r="562">
@@ -7615,7 +7615,7 @@
         <v>17.72</v>
       </c>
       <c r="J562">
-        <v>6.04</v>
+        <v>6.05</v>
       </c>
     </row>
     <row r="563">
@@ -7641,7 +7641,7 @@
         <v>43.1</v>
       </c>
       <c r="J563">
-        <v>2.62</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="564">
@@ -7667,7 +7667,7 @@
         <v>45.64</v>
       </c>
       <c r="J564">
-        <v>-2.08</v>
+        <v>-2.07</v>
       </c>
     </row>
     <row r="565">
@@ -7751,7 +7751,7 @@
         <v>31.24</v>
       </c>
       <c r="J567">
-        <v>-1.96</v>
+        <v>-2.03</v>
       </c>
     </row>
     <row r="568">
@@ -7783,7 +7783,7 @@
         <v>-31.16</v>
       </c>
       <c r="J568">
-        <v>-14.55</v>
+        <v>-14.58</v>
       </c>
     </row>
     <row r="569">
@@ -7809,7 +7809,7 @@
         <v>26.29</v>
       </c>
       <c r="J569">
-        <v>-24.63</v>
+        <v>-24.61</v>
       </c>
     </row>
     <row r="570">
@@ -7835,7 +7835,7 @@
         <v>24.37</v>
       </c>
       <c r="J570">
-        <v>-27.89</v>
+        <v>-27.85</v>
       </c>
     </row>
     <row r="571">
@@ -7867,7 +7867,7 @@
         <v>-19.61</v>
       </c>
       <c r="J571">
-        <v>-23.24</v>
+        <v>-23.23</v>
       </c>
     </row>
     <row r="572">
@@ -7919,7 +7919,7 @@
         <v>25.18</v>
       </c>
       <c r="J573">
-        <v>-17.47</v>
+        <v>-17.46</v>
       </c>
     </row>
     <row r="574">
@@ -8087,7 +8087,7 @@
         <v>39.89</v>
       </c>
       <c r="J579">
-        <v>4.33</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="580">
@@ -8119,7 +8119,7 @@
         <v>23.3</v>
       </c>
       <c r="J580">
-        <v>20.81</v>
+        <v>20.78</v>
       </c>
     </row>
     <row r="581">
@@ -8145,7 +8145,7 @@
         <v>39.8</v>
       </c>
       <c r="J581">
-        <v>24.36</v>
+        <v>24.37</v>
       </c>
     </row>
     <row r="582">
@@ -8171,7 +8171,7 @@
         <v>38.75</v>
       </c>
       <c r="J582">
-        <v>24.71</v>
+        <v>24.77</v>
       </c>
     </row>
     <row r="583">
@@ -8203,7 +8203,7 @@
         <v>49.45</v>
       </c>
       <c r="J583">
-        <v>30.92</v>
+        <v>30.93</v>
       </c>
     </row>
     <row r="584">
@@ -8229,7 +8229,7 @@
         <v>50.62</v>
       </c>
       <c r="J584">
-        <v>31.87</v>
+        <v>31.86</v>
       </c>
     </row>
     <row r="585">
@@ -8255,7 +8255,7 @@
         <v>61.67</v>
       </c>
       <c r="J585">
-        <v>33.97</v>
+        <v>33.98</v>
       </c>
     </row>
     <row r="586">
@@ -8287,7 +8287,7 @@
         <v>56.72</v>
       </c>
       <c r="J586">
-        <v>31.59</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="587">
@@ -8397,7 +8397,7 @@
         <v>43.49</v>
       </c>
       <c r="J590">
-        <v>31.41</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="591">
@@ -8423,7 +8423,7 @@
         <v>30.91</v>
       </c>
       <c r="J591">
-        <v>30.81</v>
+        <v>30.74</v>
       </c>
     </row>
     <row r="592">
@@ -8455,7 +8455,7 @@
         <v>54.5</v>
       </c>
       <c r="J592">
-        <v>30.36</v>
+        <v>30.32</v>
       </c>
     </row>
     <row r="593">
@@ -8481,7 +8481,7 @@
         <v>38.52</v>
       </c>
       <c r="J593">
-        <v>31.1</v>
+        <v>31.12</v>
       </c>
     </row>
     <row r="594">
@@ -8507,7 +8507,7 @@
         <v>36.87</v>
       </c>
       <c r="J594">
-        <v>34.05</v>
+        <v>34.12</v>
       </c>
     </row>
     <row r="595">
@@ -8539,7 +8539,7 @@
         <v>51.77</v>
       </c>
       <c r="J595">
-        <v>30.01</v>
+        <v>30.05</v>
       </c>
     </row>
     <row r="596">
@@ -8565,7 +8565,7 @@
         <v>26.95</v>
       </c>
       <c r="J596">
-        <v>23.02</v>
+        <v>22.99</v>
       </c>
     </row>
     <row r="597">
@@ -8591,7 +8591,7 @@
         <v>30.97</v>
       </c>
       <c r="J597">
-        <v>22.3</v>
+        <v>22.32</v>
       </c>
     </row>
     <row r="598">
@@ -8623,7 +8623,7 @@
         <v>42.3</v>
       </c>
       <c r="J598">
-        <v>21.96</v>
+        <v>21.97</v>
       </c>
     </row>
     <row r="599">
@@ -8675,7 +8675,7 @@
         <v>27.85</v>
       </c>
       <c r="J600">
-        <v>18.92</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="601">
@@ -8707,7 +8707,7 @@
         <v>46.15</v>
       </c>
       <c r="J601">
-        <v>29.5</v>
+        <v>29.48</v>
       </c>
     </row>
     <row r="602">
@@ -8733,7 +8733,7 @@
         <v>36.76</v>
       </c>
       <c r="J602">
-        <v>18.74</v>
+        <v>18.71</v>
       </c>
     </row>
     <row r="603">
@@ -8759,7 +8759,7 @@
         <v>43.97</v>
       </c>
       <c r="J603">
-        <v>16.94</v>
+        <v>16.87</v>
       </c>
     </row>
     <row r="604">
@@ -8791,7 +8791,7 @@
         <v>37.79</v>
       </c>
       <c r="J604">
-        <v>7.85</v>
+        <v>7.78</v>
       </c>
     </row>
     <row r="605">
@@ -8817,7 +8817,7 @@
         <v>42.47</v>
       </c>
       <c r="J605">
-        <v>-0.15</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="606">
@@ -8843,7 +8843,7 @@
         <v>42.26</v>
       </c>
       <c r="J606">
-        <v>-0.55</v>
+        <v>-0.44</v>
       </c>
     </row>
     <row r="607">
@@ -8875,7 +8875,7 @@
         <v>21.34</v>
       </c>
       <c r="J607">
-        <v>-5.99</v>
+        <v>-5.93</v>
       </c>
     </row>
     <row r="608">
@@ -8901,7 +8901,7 @@
         <v>43.1</v>
       </c>
       <c r="J608">
-        <v>-2.72</v>
+        <v>-2.75</v>
       </c>
     </row>
     <row r="609">
@@ -8927,7 +8927,7 @@
         <v>41.5</v>
       </c>
       <c r="J609">
-        <v>-4.22</v>
+        <v>-4.18</v>
       </c>
     </row>
     <row r="610">
@@ -8959,7 +8959,7 @@
         <v>14.86</v>
       </c>
       <c r="J610">
-        <v>-10.36</v>
+        <v>-10.34</v>
       </c>
     </row>
     <row r="611">
@@ -9011,7 +9011,7 @@
         <v>44.19</v>
       </c>
       <c r="J612">
-        <v>-9.83</v>
+        <v>-9.85</v>
       </c>
     </row>
     <row r="613">
@@ -9043,7 +9043,7 @@
         <v>7.6</v>
       </c>
       <c r="J613">
-        <v>-13.77</v>
+        <v>-13.8</v>
       </c>
     </row>
     <row r="614">
@@ -9069,7 +9069,7 @@
         <v>48.82</v>
       </c>
       <c r="J614">
-        <v>-15.82</v>
+        <v>-15.87</v>
       </c>
     </row>
     <row r="615">
@@ -9095,7 +9095,7 @@
         <v>43.72</v>
       </c>
       <c r="J615">
-        <v>-15.86</v>
+        <v>-15.94</v>
       </c>
     </row>
     <row r="616">
@@ -9127,7 +9127,7 @@
         <v>-1.98</v>
       </c>
       <c r="J616">
-        <v>-12.93</v>
+        <v>-13.08</v>
       </c>
     </row>
     <row r="617">
@@ -9153,7 +9153,7 @@
         <v>51.03</v>
       </c>
       <c r="J617">
-        <v>-13.02</v>
+        <v>-12.96</v>
       </c>
     </row>
     <row r="618">
@@ -9179,7 +9179,7 @@
         <v>47.72</v>
       </c>
       <c r="J618">
-        <v>-22.46</v>
+        <v>-22.32</v>
       </c>
     </row>
     <row r="619">
@@ -9211,7 +9211,7 @@
         <v>-7.1</v>
       </c>
       <c r="J619">
-        <v>-8.1</v>
+        <v>-8.01</v>
       </c>
     </row>
     <row r="620">
@@ -9263,7 +9263,7 @@
         <v>47.73</v>
       </c>
       <c r="J621">
-        <v>-10.08</v>
+        <v>-10.03</v>
       </c>
     </row>
     <row r="622">
@@ -9295,7 +9295,7 @@
         <v>-4</v>
       </c>
       <c r="J622">
-        <v>-7.99</v>
+        <v>-7.96</v>
       </c>
     </row>
     <row r="623">
@@ -9321,7 +9321,7 @@
         <v>45.56</v>
       </c>
       <c r="J623">
-        <v>-6.53</v>
+        <v>-6.52</v>
       </c>
     </row>
     <row r="624">
@@ -9347,7 +9347,7 @@
         <v>50.26</v>
       </c>
       <c r="J624">
-        <v>-7.41</v>
+        <v>-7.43</v>
       </c>
     </row>
     <row r="625">
@@ -9379,7 +9379,7 @@
         <v>-1.65</v>
       </c>
       <c r="J625">
-        <v>-11.32</v>
+        <v>-11.36</v>
       </c>
     </row>
     <row r="626">
@@ -9405,7 +9405,7 @@
         <v>38.13</v>
       </c>
       <c r="J626">
-        <v>-11.81</v>
+        <v>-11.88</v>
       </c>
     </row>
     <row r="627">
@@ -9431,7 +9431,7 @@
         <v>37.25</v>
       </c>
       <c r="J627">
-        <v>-11.77</v>
+        <v>-11.86</v>
       </c>
     </row>
     <row r="628">
@@ -9463,7 +9463,7 @@
         <v>-2.37</v>
       </c>
       <c r="J628">
-        <v>-12.04</v>
+        <v>-12.28</v>
       </c>
     </row>
     <row r="629">
@@ -9489,7 +9489,7 @@
         <v>32.24</v>
       </c>
       <c r="J629">
-        <v>-9.33</v>
+        <v>-9.3</v>
       </c>
     </row>
     <row r="630">
@@ -9515,7 +9515,7 @@
         <v>38.27</v>
       </c>
       <c r="J630">
-        <v>-7.39</v>
+        <v>-7.21</v>
       </c>
     </row>
     <row r="631">
@@ -9547,7 +9547,7 @@
         <v>0.27</v>
       </c>
       <c r="J631">
-        <v>-7.54</v>
+        <v>-7.42</v>
       </c>
     </row>
     <row r="632">
@@ -9573,7 +9573,7 @@
         <v>36.16</v>
       </c>
       <c r="J632">
-        <v>-17.85</v>
+        <v>-17.83</v>
       </c>
     </row>
     <row r="633">
@@ -9599,7 +9599,7 @@
         <v>37.28</v>
       </c>
       <c r="J633">
-        <v>-17.86</v>
+        <v>-17.78</v>
       </c>
     </row>
     <row r="634">
@@ -9631,7 +9631,7 @@
         <v>1.39</v>
       </c>
       <c r="J634">
-        <v>-4.42</v>
+        <v>-4.38</v>
       </c>
     </row>
     <row r="635">
@@ -9657,7 +9657,7 @@
         <v>38.75</v>
       </c>
       <c r="J635">
-        <v>-10.14</v>
+        <v>-10.12</v>
       </c>
     </row>
     <row r="636">
@@ -9683,7 +9683,7 @@
         <v>39.11</v>
       </c>
       <c r="J636">
-        <v>-7.28</v>
+        <v>-7.29</v>
       </c>
     </row>
     <row r="637">
@@ -9715,7 +9715,7 @@
         <v>6.41</v>
       </c>
       <c r="J637">
-        <v>7.22</v>
+        <v>7.19</v>
       </c>
     </row>
     <row r="638">
@@ -9741,7 +9741,7 @@
         <v>43.9</v>
       </c>
       <c r="J638">
-        <v>3.99</v>
+        <v>3.93</v>
       </c>
     </row>
     <row r="639">
@@ -9767,7 +9767,7 @@
         <v>43.44</v>
       </c>
       <c r="J639">
-        <v>-0.56</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="640">
@@ -9799,12 +9799,20 @@
         <v>8.79</v>
       </c>
       <c r="J640">
-        <v>4.36</v>
+        <v>4.06</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="str">
+        <v>2026-05</v>
+      </c>
+      <c r="J641">
+        <v>2.68</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J640"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J641"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>